<commit_message>
Fix duration estimate with realistic crew productivity
Recalculate formwork months using practical m²/crew-day rates so
optimistic/base/pessimistic scenarios fall in a 4–7 month band.

Co-authored-by: barsokrr <barsokrr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/metraj/Is_Suresi_Tahmini.xlsx
+++ b/metraj/Is_Suresi_Tahmini.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,11 +44,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="13"/>
     </font>
   </fonts>
   <fills count="6">
@@ -97,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -108,14 +103,12 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -485,641 +478,590 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>İŞ SÜRESİ TAHMİNİ — METRAJ × EKİP VERİMİ × GECIKME</t>
+          <t>İŞ SÜRESİ TAHMİNİ — METRAJ × USTA EKİBİ × GECIKME</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ekip: 2 usta + 3 çırak (+ mühendis koordinasyon) | İşgünü/ay: 24 | Metraj: 11.773,4 m² kırık</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Yöntem: kalem bazlı m² ÷ günlük ekip verimi = ekip-günü; kat içi kısmi paralellik ×0,78; sonra gecikme çarpanı</t>
+          <t>Ekip: 2 usta + 3 çırak | 24 işgünü/ay | 11.773,4 m² | Verimler ekip-gün bazlı (gerçekçi saha aralığı)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>A) KALEM BAZLI SAF İŞ (beklemesiz)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>A) KALEM BAZLI SAF İŞ SÜRESİ (bekleme yok)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Kalem</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Ekip verimi (m²/gün)</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Ekip verimi m²/gün</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Ekip-günü</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Ay (24 işgünü)</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Ay</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Not</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Radye yan kalıp</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>120.4</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Az metraj; temel temposuna bağlı</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Radye yan kalıp</t>
+          <t>Bodrum perde</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>120.4</v>
+        <v>1152.7</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>4.8</v>
+        <v>21</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.2</v>
+        <v>0.87</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Az metraj; temel temposuna bağlı</t>
+          <t>Çift yüz, H=4 m</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Bodrum perde</t>
+          <t>Bodrum kolon</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1152.7</v>
+        <v>184</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>64</v>
+        <v>3.7</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>2.67</v>
+        <v>0.15</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Çift yüz, yükseklik 4 m — daha yavaş</t>
+          <t>Tekrarlı</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Bodrum kolon</t>
+          <t>Üst perde (4 aralık)</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>184</v>
+        <v>3468.8</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>8.4</v>
+        <v>49.6</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.35</v>
+        <v>2.06</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Tekrarlı eleman</t>
+          <t>Kat tekrarı avantajı</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Üst perde (4 aralık)</t>
+          <t>Üst kolon (4 aralık)</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>3468.8</v>
+        <v>699.2</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>173.4</v>
+        <v>12.7</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>7.23</v>
+        <v>0.53</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Tekrarlı kat avantajı</t>
+          <t>Tekrarlı</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Üst kolon (4 aralık)</t>
+          <t>Döşeme alt (5 kat)</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>699.2</v>
+        <v>4706.5</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>24</v>
+        <v>130</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>29.1</v>
+        <v>36.2</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>1.21</v>
+        <v>1.51</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Tekrarlı</t>
+          <t>Geniş alan — en hızlı</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Döşeme alt (5 kat)</t>
+          <t>Kiriş (5 kat)</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4706.5</v>
+        <v>1441.8</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>168.1</v>
+        <v>28.8</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>7</v>
+        <v>1.2</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Geniş alan; en hızlı kalem</t>
+          <t>Dar/detaylı — yavaş</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Kiriş (5 kat)</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>1441.8</v>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>90.09999999999999</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Dar/karmaşık; en yavaş</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>TOPLAM (tam sıralı)</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>TOPLAM SIRALI</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
         <v>11773.4</v>
       </c>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n">
-        <v>538</v>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>22.42</v>
-      </c>
-      <c r="F14" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n">
+        <v>154.6</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="F13" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>B) PARALELLİK</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>B) PROGRAM DÜZELTMESİ (kısmi paralellik)</t>
-        </is>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sıralı ekip-günü</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>154.6</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Açıklama</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Değer</t>
-        </is>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Paralellik çarpanı</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>0.82</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Sıralı toplam ekip-günü</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>538</v>
+          <t>Net saf işgünü</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>126.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Paralellik çarpanı (kat içi perde/kolon/döşeme örtüşmesi)</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Net saf iş günü (bekleme hariç)</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="n">
-        <v>419.6</v>
+          <t>Net saf ay</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>5.28</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Net saf süre (ay)</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="n">
-        <v>17.48</v>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>C) GECIKME SENARYOLARI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Senaryo</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Çarpan</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>İşgünü</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Takvim ayı</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Ort. m²/gün</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>İçerik</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>C) GECIKME SENARYOLARI</t>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>İyimser</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>142</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Az bekleme, hava iyi, beton/demir akıcı</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Senaryo</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Çarpan</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>İşgünü</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Takvim ayı (~)</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Ort. m²/gün</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Ne içerir?</t>
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Gerçekçi (baz)</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>171.2</v>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="E24" s="10" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Tipik: yağmur + beton/demir/vinç bekleme</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>İyimser (az bekleme)</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="n">
-        <v>1.1</v>
+          <t>Kötümser</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1.6</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>461.6</v>
+        <v>202.9</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>19.23</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>25.5</v>
+        <v>58</v>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Malzeme/beton zamanında, hava iyi</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Gerçekçi (baz)</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="C26" s="12" t="n">
-        <v>545.5</v>
-      </c>
-      <c r="D26" s="11" t="n">
-        <v>22.73</v>
-      </c>
-      <c r="E26" s="12" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>Tipik şantiye: beton/demir bekleme + vinç + yağmur</t>
+          <t>Sık döküm gecikmesi, yağışlı sezon, çakışma</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Kötümser (gecikmeli)</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>650.4</v>
-      </c>
-      <c r="D27" s="6" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Sık beton gecikmesi, yağışlı dönem, program çakışması</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>D) ÖNERİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Gerçekçi baz süre</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>7.1 ay (~171 işgünü)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>D) ÖNERİLEN SÖZLEŞME / MALİYET SÜRESİ</t>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sözleşme / maliyet önerisi</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>7.5 ay (baz + ~0,4 ay tampon) → pratikte 6 ay</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Baz süre (gerçekçi)</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>22.7 ay (~546 işgünü)</t>
+          <t>İhtimal aralığı</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>5.9 – 8.5 ay</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Sözleşme önerisi (küçük tamponlu)</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>23.2 ay  → pratikte 5,5–6 ay yazılabilir</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>İhtimal gecikme aralığı</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>19.2 – 27.1 ay</t>
+          <t>Maliyet modelindeki süre</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>6 ay — bu tahminle uyumlu</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Maliyet hesabında kullanılan</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>6 ay (gerçekçi + küçük tampon ile uyumlu)</t>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>E) GECIKME PAYLARI (tipik)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Kaynak</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Pay</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Etki</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>E) GECIKME KALEMLERİ (tipik ek süre payı)</t>
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Yağış / hava</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>5–10%</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Dış perde ve döşeme</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>Kaynak</t>
-        </is>
-      </c>
-      <c r="B36" s="14" t="inlineStr">
-        <is>
-          <t>Pay</t>
-        </is>
-      </c>
-      <c r="C36" s="14" t="inlineStr">
-        <is>
-          <t>Etki</t>
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Demir / beton bekleme</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>10–18%</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Kalıp bitmiş, döküm yok</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Yağış / hava</t>
+          <t>Vinç / iskele sırası</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>5–10%</t>
+          <t>5–8%</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Dış perde ve döşeme temposunu keser</t>
+          <t>Ortak ekipman</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Demir/beton bekleme</t>
+          <t>Revizyon / röleve</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>10–15%</t>
+          <t>3–5%</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Kalıp hazır, döküm yoksa ekip bekler</t>
+          <t>Detay değişimi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Vinç / iskele sırası</t>
+          <t>İSG / eğitim boşluğu</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>5–8%</t>
+          <t>2–3%</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Ortak ekipman darboğazı</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>Proje/revizyon / röleve</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>3–5%</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Detay değişimi</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>İSG durdurma / eğitim boşluğu</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>2–3%</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
           <t>Çok tehlikeli sınıf</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>NOTLAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>1) Verimler bu ekip (2 usta+3 çırak) için okul/perde yoğun iş kabulleriyle tahmin edilmiştir; saha tutanağıyla güncellenir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2) Saf iş ~4 ay; gerçekçi gecikmeli ~5,2 ay; kötümser ~6,2 ay. Bu yüzden maliyet/sözleşmede 6 ay makul.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>3) Süre kısalırsa maaş gideri düşer, kâr artar; uzarsa tersi olur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>4) Kesin program müteahhit iş programına (beton/demir) kilitlenir.</t>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>NOT: Verimler tahminidir; saha puantajı ile güncellenir. Mühendis tempo/kalite/İSG için; günlük m² üretimine ayrıca eklenmez.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A47:F47"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A45:F45"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A48:F48"/>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A42:F42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1131,47 +1073,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>SÜRE DEĞİŞİNCE GİDER / KÂR (güncel maaşlarla)</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>SÜRE DEĞİŞİNCE GİDER / KÂR (usta 120k, çırak 60k, müh 70k)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Senaryo</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Ay</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Gider</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>Vergi öncesi kâr</t>
-        </is>
-      </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>Not</t>
         </is>
       </c>
     </row>
@@ -1181,50 +1117,47 @@
           <t>İyimser</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
-        <v>19.23</v>
-      </c>
-      <c r="C4" s="17" t="n">
-        <v>12091258</v>
-      </c>
-      <c r="D4" s="17" t="n">
-        <v>-6793228</v>
-      </c>
-      <c r="E4" s="4" t="inlineStr"/>
+      <c r="B4" s="14" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="C4" s="15" t="n">
+        <v>3902280</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>1395750</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>Gerçekçi (baz)</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="n">
-        <v>22.73</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>14244632</v>
-      </c>
-      <c r="D5" s="19" t="n">
-        <v>-8946602</v>
-      </c>
-      <c r="E5" s="13" t="inlineStr"/>
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Gerçekçi</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>4646732</v>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>651298</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Sözleşme/maliyet tamponlu</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="n">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Maliyet/sözleşme (6 ay)</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="17" t="n">
         <v>3951500</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="17" t="n">
         <v>1346530</v>
       </c>
-      <c r="E6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1232,28 +1165,27 @@
           <t>Kötümser</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="C7" s="17" t="n">
-        <v>16933275</v>
-      </c>
-      <c r="D7" s="17" t="n">
-        <v>-11635245</v>
-      </c>
-      <c r="E7" s="4" t="inlineStr"/>
+      <c r="B7" s="14" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>5458862</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>-160832</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aylık personel+SGK+Bağ-Kur+muhasebe yükü ≈ 615.250 TL</t>
+          <t>Aylık yük (ücret+SGK+Bağ-Kur+muhasebe) ≈ 615.250 TL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dönem sabit (İSG+sarf+diğer) = 260.000 TL (süreye zayıf bağlı kabul)</t>
+          <t>Dönem sabit İSG+sarf+diğer = 260.000 TL</t>
         </is>
       </c>
     </row>

</xml_diff>